<commit_message>
nyoba ADI dan CV2
</commit_message>
<xml_diff>
--- a/data_output/03_K_EVALUATION_DBI.xlsx
+++ b/data_output/03_K_EVALUATION_DBI.xlsx
@@ -727,7 +727,7 @@
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>60.4894886856584</v>
+        <v>60.48948868565841</v>
       </c>
       <c r="D12" t="n">
         <v>1.013750062291383</v>
@@ -777,7 +777,7 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>45.02581389054694</v>
+        <v>45.02581389054693</v>
       </c>
       <c r="D14" t="n">
         <v>0.9455431039178561</v>
@@ -802,7 +802,7 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>39.70679283120539</v>
+        <v>39.70679283120538</v>
       </c>
       <c r="D15" t="n">
         <v>0.9102931252340507</v>
@@ -827,7 +827,7 @@
         <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>2574.773304386981</v>
+        <v>2574.77330438698</v>
       </c>
       <c r="D16" t="n">
         <v>0.7435418930393753</v>
@@ -1052,7 +1052,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>17.57995370120434</v>
+        <v>17.57995370120435</v>
       </c>
       <c r="D25" t="n">
         <v>0.6549248415596544</v>
@@ -1077,7 +1077,7 @@
         <v>5</v>
       </c>
       <c r="C26" t="n">
-        <v>12.48913443163634</v>
+        <v>12.48913443163633</v>
       </c>
       <c r="D26" t="n">
         <v>0.6780759443353374</v>
@@ -1102,7 +1102,7 @@
         <v>6</v>
       </c>
       <c r="C27" t="n">
-        <v>9.951790670295649</v>
+        <v>9.951790670295651</v>
       </c>
       <c r="D27" t="n">
         <v>0.652975848340566</v>
@@ -1152,7 +1152,7 @@
         <v>8</v>
       </c>
       <c r="C29" t="n">
-        <v>7.230948886520392</v>
+        <v>7.23094888652039</v>
       </c>
       <c r="D29" t="n">
         <v>0.7121198723833853</v>
@@ -1428,7 +1428,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>39.70679283120539</v>
+        <v>39.70679283120538</v>
       </c>
       <c r="D3" t="n">
         <v>0.9102931252340507</v>

</xml_diff>

<commit_message>
bener ADI + CV2
</commit_message>
<xml_diff>
--- a/data_output/03_K_EVALUATION_DBI.xlsx
+++ b/data_output/03_K_EVALUATION_DBI.xlsx
@@ -577,7 +577,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>903.5182740522188</v>
+        <v>903.518274052219</v>
       </c>
       <c r="D6" t="n">
         <v>1.013300513349807</v>
@@ -727,7 +727,7 @@
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>60.4894886856584</v>
+        <v>60.48948868565841</v>
       </c>
       <c r="D12" t="n">
         <v>1.013750062291383</v>
@@ -752,7 +752,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>52.65678071523887</v>
+        <v>52.65678071523885</v>
       </c>
       <c r="D13" t="n">
         <v>1.094887946497466</v>
@@ -777,7 +777,7 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>45.02581389054694</v>
+        <v>45.02581389054693</v>
       </c>
       <c r="D14" t="n">
         <v>0.9455431039178561</v>
@@ -802,7 +802,7 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>39.70679283120539</v>
+        <v>39.70679283120538</v>
       </c>
       <c r="D15" t="n">
         <v>0.9102931252340507</v>
@@ -902,7 +902,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>894.8930522099873</v>
+        <v>894.8930522099872</v>
       </c>
       <c r="D19" t="n">
         <v>0.6648785993929051</v>
@@ -1052,7 +1052,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>17.57995370120434</v>
+        <v>17.57995370120435</v>
       </c>
       <c r="D25" t="n">
         <v>0.6549248415596544</v>
@@ -1152,7 +1152,7 @@
         <v>8</v>
       </c>
       <c r="C29" t="n">
-        <v>7.230948886520392</v>
+        <v>7.23094888652039</v>
       </c>
       <c r="D29" t="n">
         <v>0.7121198723833853</v>
@@ -1428,7 +1428,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>39.70679283120539</v>
+        <v>39.70679283120538</v>
       </c>
       <c r="D3" t="n">
         <v>0.9102931252340507</v>

</xml_diff>

<commit_message>
only ADI + CV2
</commit_message>
<xml_diff>
--- a/data_output/03_K_EVALUATION_DBI.xlsx
+++ b/data_output/03_K_EVALUATION_DBI.xlsx
@@ -477,19 +477,19 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>2343.786681897217</v>
+        <v>1148.640186135502</v>
       </c>
       <c r="D2" t="n">
-        <v>1.072992952240863</v>
+        <v>0.7034174160993338</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3789236987737462</v>
+        <v>0.6380402368280619</v>
       </c>
       <c r="F2" t="n">
-        <v>927.9525635173266</v>
+        <v>1791.145891822144</v>
       </c>
       <c r="G2" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="3">
@@ -502,19 +502,19 @@
         <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>1637.469502495703</v>
+        <v>671.9428700783047</v>
       </c>
       <c r="D3" t="n">
-        <v>1.024780734538243</v>
+        <v>0.7317022745812723</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3544801051775885</v>
+        <v>0.6021952263868707</v>
       </c>
       <c r="F3" t="n">
-        <v>949.3773485412911</v>
+        <v>2004.742231025668</v>
       </c>
       <c r="G3" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="4">
@@ -527,19 +527,19 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>1305.0497558203</v>
+        <v>474.0110678793847</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9320287181319101</v>
+        <v>0.7567474087321098</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3327849980318259</v>
+        <v>0.5979419239196372</v>
       </c>
       <c r="F4" t="n">
-        <v>905.9578687646278</v>
+        <v>2079.392508987993</v>
       </c>
       <c r="G4" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="5">
@@ -552,19 +552,19 @@
         <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>1073.80615930946</v>
+        <v>383.8412867767072</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9465543781342097</v>
+        <v>0.8080320124278897</v>
       </c>
       <c r="E5" t="n">
-        <v>0.332972869753754</v>
+        <v>0.5782779029385668</v>
       </c>
       <c r="F5" t="n">
-        <v>896.3876808337427</v>
+        <v>2002.984244741067</v>
       </c>
       <c r="G5" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="6">
@@ -577,19 +577,19 @@
         <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>903.518274052219</v>
+        <v>306.7557683540558</v>
       </c>
       <c r="D6" t="n">
-        <v>1.013300513349807</v>
+        <v>0.7058153748725958</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3303842143353738</v>
+        <v>0.6474704039118676</v>
       </c>
       <c r="F6" t="n">
-        <v>901.4531213493976</v>
+        <v>2070.701594640102</v>
       </c>
       <c r="G6" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="7">
@@ -602,19 +602,19 @@
         <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>790.1950468876809</v>
+        <v>245.3787369845955</v>
       </c>
       <c r="D7" t="n">
-        <v>0.974205573067786</v>
+        <v>0.7079860071700833</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3312560681417659</v>
+        <v>0.6544579762222865</v>
       </c>
       <c r="F7" t="n">
-        <v>889.868132279217</v>
+        <v>2211.247957702986</v>
       </c>
       <c r="G7" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="8">
@@ -627,19 +627,19 @@
         <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>722.0475933325158</v>
+        <v>207.1250517021849</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9832094627581502</v>
+        <v>0.6614119260840338</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3265657260969269</v>
+        <v>0.6569899929289034</v>
       </c>
       <c r="F8" t="n">
-        <v>851.898172554434</v>
+        <v>2278.920842316035</v>
       </c>
       <c r="G8" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="9">
@@ -652,19 +652,19 @@
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>133.0310371977093</v>
+        <v>28.45225440259275</v>
       </c>
       <c r="D9" t="n">
-        <v>1.096195672452495</v>
+        <v>0.5964873399479999</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3733051030938709</v>
+        <v>0.6407572015382345</v>
       </c>
       <c r="F9" t="n">
-        <v>951.4661146539287</v>
+        <v>2858.109076114852</v>
       </c>
       <c r="G9" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="10">
@@ -677,19 +677,19 @@
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>90.93400280272579</v>
+        <v>16.48084405696105</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9650001835284433</v>
+        <v>0.6771663659907866</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3832939112914902</v>
+        <v>0.6097505876593239</v>
       </c>
       <c r="F10" t="n">
-        <v>1002.14239528811</v>
+        <v>2951.56844992709</v>
       </c>
       <c r="G10" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="11">
@@ -702,19 +702,19 @@
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>72.02309563756953</v>
+        <v>11.81035831179882</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9589512574858545</v>
+        <v>0.7576173048182246</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3526809307468047</v>
+        <v>0.5964993999475097</v>
       </c>
       <c r="F11" t="n">
-        <v>958.7578589971514</v>
+        <v>2920.180409297017</v>
       </c>
       <c r="G11" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="12">
@@ -727,19 +727,19 @@
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>60.48948868565841</v>
+        <v>9.302227530498406</v>
       </c>
       <c r="D12" t="n">
-        <v>1.013750062291383</v>
+        <v>0.7226956684046515</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3185641003007509</v>
+        <v>0.6318236378939948</v>
       </c>
       <c r="F12" t="n">
-        <v>918.5919318386593</v>
+        <v>2868.699276916</v>
       </c>
       <c r="G12" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="13">
@@ -752,19 +752,19 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>52.65678071523885</v>
+        <v>7.074549623175549</v>
       </c>
       <c r="D13" t="n">
-        <v>1.094887946497466</v>
+        <v>0.7000227472655149</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3084376261047577</v>
+        <v>0.6484933539357631</v>
       </c>
       <c r="F13" t="n">
-        <v>882.8776252603616</v>
+        <v>3099.491013719199</v>
       </c>
       <c r="G13" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="14">
@@ -777,19 +777,19 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>45.02581389054693</v>
+        <v>5.919858785356674</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9455431039178561</v>
+        <v>0.698817285480354</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3245349560431947</v>
+        <v>0.6592339144351974</v>
       </c>
       <c r="F14" t="n">
-        <v>897.0859292929745</v>
+        <v>3127.804429244224</v>
       </c>
       <c r="G14" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="15">
@@ -802,19 +802,19 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>39.70679283120538</v>
+        <v>4.933440147835765</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9102931252340507</v>
+        <v>0.7105499757482725</v>
       </c>
       <c r="E15" t="n">
-        <v>0.321856365026715</v>
+        <v>0.6601158518605439</v>
       </c>
       <c r="F15" t="n">
-        <v>896.5353046440688</v>
+        <v>3252.717998377307</v>
       </c>
       <c r="G15" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="16">
@@ -827,19 +827,19 @@
         <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>2574.773304386981</v>
+        <v>1362.504696605515</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7435418930393753</v>
+        <v>0.4321825649567547</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7614705006883822</v>
+        <v>0.6555550707455412</v>
       </c>
       <c r="F16" t="n">
-        <v>725.7472318821328</v>
+        <v>1299.667965152938</v>
       </c>
       <c r="G16" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="17">
@@ -852,19 +852,19 @@
         <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>1606.696849679994</v>
+        <v>662.1932643312161</v>
       </c>
       <c r="D17" t="n">
-        <v>0.6961768783969294</v>
+        <v>0.5079118774289985</v>
       </c>
       <c r="E17" t="n">
-        <v>0.525617556196998</v>
+        <v>0.7247959574312186</v>
       </c>
       <c r="F17" t="n">
-        <v>980.2518402139941</v>
+        <v>2044.115641824478</v>
       </c>
       <c r="G17" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="18">
@@ -877,19 +877,19 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1131.714066935433</v>
+        <v>412.7421150882933</v>
       </c>
       <c r="D18" t="n">
-        <v>0.5312591726852109</v>
+        <v>0.4219089895499252</v>
       </c>
       <c r="E18" t="n">
-        <v>0.5298667733772454</v>
+        <v>0.7281729917781605</v>
       </c>
       <c r="F18" t="n">
-        <v>1112.316864299002</v>
+        <v>2454.271031813475</v>
       </c>
       <c r="G18" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="19">
@@ -902,19 +902,19 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>894.8930522099872</v>
+        <v>247.3293731147099</v>
       </c>
       <c r="D19" t="n">
-        <v>0.6648785993929051</v>
+        <v>0.4678546340469087</v>
       </c>
       <c r="E19" t="n">
-        <v>0.5403089156129522</v>
+        <v>0.7052019605213105</v>
       </c>
       <c r="F19" t="n">
-        <v>1141.72539440143</v>
+        <v>3293.067667615018</v>
       </c>
       <c r="G19" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="20">
@@ -927,19 +927,19 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>718.061489817884</v>
+        <v>158.2565554078886</v>
       </c>
       <c r="D20" t="n">
-        <v>0.6744711013465983</v>
+        <v>0.4864509443328934</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4760183920694584</v>
+        <v>0.7077793279322626</v>
       </c>
       <c r="F20" t="n">
-        <v>1202.566499423626</v>
+        <v>4264.459356237017</v>
       </c>
       <c r="G20" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="21">
@@ -952,19 +952,19 @@
         <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>590.7322190464478</v>
+        <v>108.1671780301969</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6074920608666784</v>
+        <v>0.4871007377633259</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4803844089965166</v>
+        <v>0.7151670437018306</v>
       </c>
       <c r="F21" t="n">
-        <v>1264.714723933976</v>
+        <v>5298.490848381786</v>
       </c>
       <c r="G21" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="22">
@@ -977,19 +977,19 @@
         <v>8</v>
       </c>
       <c r="C22" t="n">
-        <v>491.5102342719914</v>
+        <v>84.1073718595912</v>
       </c>
       <c r="D22" t="n">
-        <v>0.6787773810231419</v>
+        <v>0.561159313570525</v>
       </c>
       <c r="E22" t="n">
-        <v>0.4886450628152035</v>
+        <v>0.7092624762076667</v>
       </c>
       <c r="F22" t="n">
-        <v>1339.918761549079</v>
+        <v>5890.865941028016</v>
       </c>
       <c r="G22" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="23">
@@ -1002,19 +1002,19 @@
         <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>41.47086099086746</v>
+        <v>30.66661277735404</v>
       </c>
       <c r="D23" t="n">
-        <v>0.5719910452087451</v>
+        <v>0.2102506026705716</v>
       </c>
       <c r="E23" t="n">
-        <v>0.5919146977229509</v>
+        <v>0.8123717714369675</v>
       </c>
       <c r="F23" t="n">
-        <v>2939.772747377972</v>
+        <v>8918.678313108905</v>
       </c>
       <c r="G23" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="24">
@@ -1027,19 +1027,19 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>24.08270110298326</v>
+        <v>9.967809059302205</v>
       </c>
       <c r="D24" t="n">
-        <v>0.6349567689270076</v>
+        <v>0.3923073107269741</v>
       </c>
       <c r="E24" t="n">
-        <v>0.5447840014680624</v>
+        <v>0.7761895953316804</v>
       </c>
       <c r="F24" t="n">
-        <v>3007.60027545888</v>
+        <v>15099.46880022753</v>
       </c>
       <c r="G24" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="25">
@@ -1052,19 +1052,19 @@
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>17.57995370120435</v>
+        <v>6.296345917817116</v>
       </c>
       <c r="D25" t="n">
-        <v>0.6549248415596544</v>
+        <v>0.4552305494722576</v>
       </c>
       <c r="E25" t="n">
-        <v>0.5282484526412602</v>
+        <v>0.7504923205471863</v>
       </c>
       <c r="F25" t="n">
-        <v>2907.906491838825</v>
+        <v>16184.2470732317</v>
       </c>
       <c r="G25" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="26">
@@ -1077,19 +1077,19 @@
         <v>5</v>
       </c>
       <c r="C26" t="n">
-        <v>12.48913443163634</v>
+        <v>4.003815311841544</v>
       </c>
       <c r="D26" t="n">
-        <v>0.6780759443353374</v>
+        <v>0.500769470659252</v>
       </c>
       <c r="E26" t="n">
-        <v>0.5526824116978944</v>
+        <v>0.7580210800405238</v>
       </c>
       <c r="F26" t="n">
-        <v>3202.681269869673</v>
+        <v>19265.46708591973</v>
       </c>
       <c r="G26" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="27">
@@ -1102,19 +1102,19 @@
         <v>6</v>
       </c>
       <c r="C27" t="n">
-        <v>9.951790670295649</v>
+        <v>2.908480999763507</v>
       </c>
       <c r="D27" t="n">
-        <v>0.652975848340566</v>
+        <v>0.5361809577193704</v>
       </c>
       <c r="E27" t="n">
-        <v>0.5282425304308055</v>
+        <v>0.7398324673917163</v>
       </c>
       <c r="F27" t="n">
-        <v>3280.120249322243</v>
+        <v>21304.33804431949</v>
       </c>
       <c r="G27" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="28">
@@ -1127,19 +1127,19 @@
         <v>7</v>
       </c>
       <c r="C28" t="n">
-        <v>8.487686106285802</v>
+        <v>1.993307183764497</v>
       </c>
       <c r="D28" t="n">
-        <v>0.7224299773725706</v>
+        <v>0.4763277475353345</v>
       </c>
       <c r="E28" t="n">
-        <v>0.537343924070138</v>
+        <v>0.7458392556455353</v>
       </c>
       <c r="F28" t="n">
-        <v>3240.497853891739</v>
+        <v>25983.95071987797</v>
       </c>
       <c r="G28" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="29">
@@ -1152,19 +1152,19 @@
         <v>8</v>
       </c>
       <c r="C29" t="n">
-        <v>7.23094888652039</v>
+        <v>1.57140636616082</v>
       </c>
       <c r="D29" t="n">
-        <v>0.7121198723833853</v>
+        <v>0.5291053257105305</v>
       </c>
       <c r="E29" t="n">
-        <v>0.5151217405421817</v>
+        <v>0.7337440735377563</v>
       </c>
       <c r="F29" t="n">
-        <v>3290.712913745401</v>
+        <v>28289.53661728291</v>
       </c>
       <c r="G29" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="30">
@@ -1177,19 +1177,19 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>5.929917029434037e+21</v>
+        <v>30576171.55513669</v>
       </c>
       <c r="D30" t="n">
-        <v>0.3821553068367418</v>
+        <v>0.1912833545711593</v>
       </c>
       <c r="E30" t="n">
-        <v>0.9202183932111728</v>
+        <v>0.8310419754592192</v>
       </c>
       <c r="F30" t="n">
-        <v>2996.221017599002</v>
+        <v>10687.05119476751</v>
       </c>
       <c r="G30" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="31">
@@ -1202,19 +1202,19 @@
         <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>2.997497075905267e+21</v>
+        <v>6230755.65010175</v>
       </c>
       <c r="D31" t="n">
-        <v>0.4880786964334796</v>
+        <v>0.3295976416765082</v>
       </c>
       <c r="E31" t="n">
-        <v>0.869456834987917</v>
+        <v>0.8240351955266232</v>
       </c>
       <c r="F31" t="n">
-        <v>3609.578045369726</v>
+        <v>28818.63655617612</v>
       </c>
       <c r="G31" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="32">
@@ -1227,19 +1227,19 @@
         <v>4</v>
       </c>
       <c r="C32" t="n">
-        <v>1.52346538805228e+21</v>
+        <v>2119232.476899426</v>
       </c>
       <c r="D32" t="n">
-        <v>0.4579631205168296</v>
+        <v>0.3093965355022695</v>
       </c>
       <c r="E32" t="n">
-        <v>0.8495107993967973</v>
+        <v>0.8304575162121144</v>
       </c>
       <c r="F32" t="n">
-        <v>5158.12738291785</v>
+        <v>57309.55021332813</v>
       </c>
       <c r="G32" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="33">
@@ -1252,19 +1252,19 @@
         <v>5</v>
       </c>
       <c r="C33" t="n">
-        <v>1.057319912098675e+21</v>
+        <v>824715.6774871821</v>
       </c>
       <c r="D33" t="n">
-        <v>0.4800003107704686</v>
+        <v>0.3336074807847515</v>
       </c>
       <c r="E33" t="n">
-        <v>0.8018984018139508</v>
+        <v>0.8321857549018241</v>
       </c>
       <c r="F33" t="n">
-        <v>5715.7701608126</v>
+        <v>110891.3182470198</v>
       </c>
       <c r="G33" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="34">
@@ -1277,19 +1277,19 @@
         <v>6</v>
       </c>
       <c r="C34" t="n">
-        <v>6.618377790259313e+20</v>
+        <v>408811.1984657464</v>
       </c>
       <c r="D34" t="n">
-        <v>0.4803917848769266</v>
+        <v>0.2944830235290374</v>
       </c>
       <c r="E34" t="n">
-        <v>0.8029357167307758</v>
+        <v>0.8499586249766651</v>
       </c>
       <c r="F34" t="n">
-        <v>7457.460658414732</v>
+        <v>179103.3491151219</v>
       </c>
       <c r="G34" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="35">
@@ -1302,19 +1302,19 @@
         <v>7</v>
       </c>
       <c r="C35" t="n">
-        <v>4.910991085222902e+20</v>
+        <v>207745.270950346</v>
       </c>
       <c r="D35" t="n">
-        <v>0.4777458861061524</v>
+        <v>0.3203799710508312</v>
       </c>
       <c r="E35" t="n">
-        <v>0.7796783734203883</v>
+        <v>0.8456879148398341</v>
       </c>
       <c r="F35" t="n">
-        <v>8445.350462257669</v>
+        <v>293702.3712082088</v>
       </c>
       <c r="G35" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="36">
@@ -1327,19 +1327,19 @@
         <v>8</v>
       </c>
       <c r="C36" t="n">
-        <v>3.754786455949637e+20</v>
+        <v>126060.7502422596</v>
       </c>
       <c r="D36" t="n">
-        <v>0.4765865745963469</v>
+        <v>0.3089820708385294</v>
       </c>
       <c r="E36" t="n">
-        <v>0.7802070786461784</v>
+        <v>0.8493648169965379</v>
       </c>
       <c r="F36" t="n">
-        <v>9518.823805126714</v>
+        <v>414682.6176928062</v>
       </c>
       <c r="G36" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
   </sheetData>
@@ -1400,22 +1400,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1305.0497558203</v>
+        <v>207.1250517021849</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9320287181319101</v>
+        <v>0.6614119260840338</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3327849980318259</v>
+        <v>0.6569899929289034</v>
       </c>
       <c r="F2" t="n">
-        <v>905.9578687646278</v>
+        <v>2278.920842316035</v>
       </c>
       <c r="G2" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="3">
@@ -1425,22 +1425,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>39.70679283120538</v>
+        <v>28.45225440259275</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9102931252340507</v>
+        <v>0.5964873399479999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.321856365026715</v>
+        <v>0.6407572015382345</v>
       </c>
       <c r="F3" t="n">
-        <v>896.5353046440688</v>
+        <v>2858.109076114852</v>
       </c>
       <c r="G3" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="4">
@@ -1453,19 +1453,19 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>1131.714066935433</v>
+        <v>412.7421150882933</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5312591726852109</v>
+        <v>0.4219089895499252</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5298667733772454</v>
+        <v>0.7281729917781605</v>
       </c>
       <c r="F4" t="n">
-        <v>1112.316864299002</v>
+        <v>2454.271031813475</v>
       </c>
       <c r="G4" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="5">
@@ -1478,19 +1478,19 @@
         <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>41.47086099086746</v>
+        <v>30.66661277735404</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5719910452087451</v>
+        <v>0.2102506026705716</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5919146977229509</v>
+        <v>0.8123717714369675</v>
       </c>
       <c r="F5" t="n">
-        <v>2939.772747377972</v>
+        <v>8918.678313108905</v>
       </c>
       <c r="G5" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="6">
@@ -1503,19 +1503,19 @@
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>5.929917029434037e+21</v>
+        <v>30576171.55513669</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3821553068367418</v>
+        <v>0.1912833545711593</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9202183932111728</v>
+        <v>0.8310419754592192</v>
       </c>
       <c r="F6" t="n">
-        <v>2996.221017599002</v>
+        <v>10687.05119476751</v>
       </c>
       <c r="G6" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
   </sheetData>
@@ -1576,22 +1576,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1305.0497558203</v>
+        <v>207.1250517021849</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9320287181319101</v>
+        <v>0.6614119260840338</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3327849980318259</v>
+        <v>0.6569899929289034</v>
       </c>
       <c r="F2" t="n">
-        <v>905.9578687646278</v>
+        <v>2278.920842316035</v>
       </c>
       <c r="G2" t="n">
-        <v>1328</v>
+        <v>1342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>